<commit_message>
Mise a jour automatique de la collection et de la page Wanted
</commit_message>
<xml_diff>
--- a/01_Liste achat.xlsx
+++ b/01_Liste achat.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PHILIPPE\Desktop\Sauvegarde vinyles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE4F7E93-0698-4858-8EDA-77928EE43F8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{486D73D2-7C67-4118-831A-320D1441B89A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="804">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1219" uniqueCount="804">
   <si>
     <t>Artistes / Titres</t>
   </si>
@@ -3316,12 +3316,12 @@
       <c r="I2" s="19"/>
       <c r="J2" s="11">
         <f>SUM(I3:I560)</f>
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="K2" s="20"/>
       <c r="L2" s="12">
         <f>H2-J2</f>
-        <v>213</v>
+        <v>206</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
@@ -3431,18 +3431,20 @@
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="66" t="s">
+      <c r="A6" s="4" t="s">
         <v>431</v>
       </c>
-      <c r="B6" s="67"/>
-      <c r="C6" s="68"/>
-      <c r="D6" s="69" t="s">
+      <c r="B6" s="1"/>
+      <c r="C6" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="13" t="s">
         <v>430</v>
       </c>
-      <c r="E6" s="70">
+      <c r="E6" s="37">
         <v>11</v>
       </c>
-      <c r="F6" s="77" t="s">
+      <c r="F6" s="54" t="s">
         <v>550</v>
       </c>
       <c r="G6" s="21">
@@ -3452,7 +3454,7 @@
       <c r="H6" s="22"/>
       <c r="I6" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J6" s="24"/>
       <c r="K6" s="25"/>
@@ -3467,18 +3469,20 @@
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="66" t="s">
+      <c r="A7" s="4" t="s">
         <v>552</v>
       </c>
-      <c r="B7" s="67"/>
-      <c r="C7" s="68"/>
-      <c r="D7" s="69" t="s">
+      <c r="B7" s="1"/>
+      <c r="C7" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="13" t="s">
         <v>430</v>
       </c>
-      <c r="E7" s="70">
+      <c r="E7" s="37">
         <v>13.5</v>
       </c>
-      <c r="F7" s="77" t="s">
+      <c r="F7" s="54" t="s">
         <v>551</v>
       </c>
       <c r="G7" s="21">
@@ -3488,7 +3492,7 @@
       <c r="H7" s="22"/>
       <c r="I7" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J7" s="24"/>
       <c r="K7" s="25"/>
@@ -3503,18 +3507,20 @@
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="66" t="s">
+      <c r="A8" s="4" t="s">
         <v>536</v>
       </c>
-      <c r="B8" s="67"/>
-      <c r="C8" s="68"/>
-      <c r="D8" s="69" t="s">
+      <c r="B8" s="1"/>
+      <c r="C8" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="13" t="s">
         <v>430</v>
       </c>
-      <c r="E8" s="70">
+      <c r="E8" s="37">
         <v>12</v>
       </c>
-      <c r="F8" s="77" t="s">
+      <c r="F8" s="54" t="s">
         <v>553</v>
       </c>
       <c r="G8" s="21">
@@ -3524,7 +3530,7 @@
       <c r="H8" s="22"/>
       <c r="I8" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8" s="24"/>
       <c r="K8" s="25"/>
@@ -3575,18 +3581,20 @@
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="66" t="s">
+      <c r="A10" s="4" t="s">
         <v>538</v>
       </c>
-      <c r="B10" s="67"/>
-      <c r="C10" s="68"/>
-      <c r="D10" s="69" t="s">
+      <c r="B10" s="1"/>
+      <c r="C10" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D10" s="13" t="s">
         <v>430</v>
       </c>
-      <c r="E10" s="70">
+      <c r="E10" s="37">
         <v>29</v>
       </c>
-      <c r="F10" s="77" t="s">
+      <c r="F10" s="54" t="s">
         <v>555</v>
       </c>
       <c r="G10" s="21">
@@ -3596,25 +3604,27 @@
       <c r="H10" s="22"/>
       <c r="I10" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10" s="24"/>
       <c r="K10" s="25"/>
       <c r="L10" s="24"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="66" t="s">
+      <c r="A11" s="4" t="s">
         <v>539</v>
       </c>
-      <c r="B11" s="67"/>
-      <c r="C11" s="68"/>
-      <c r="D11" s="69" t="s">
+      <c r="B11" s="1"/>
+      <c r="C11" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" s="13" t="s">
         <v>430</v>
       </c>
-      <c r="E11" s="70">
+      <c r="E11" s="37">
         <v>15</v>
       </c>
-      <c r="F11" s="77" t="s">
+      <c r="F11" s="54" t="s">
         <v>556</v>
       </c>
       <c r="G11" s="21">
@@ -3624,7 +3634,7 @@
       <c r="H11" s="22"/>
       <c r="I11" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J11" s="24"/>
       <c r="K11" s="25"/>
@@ -3639,18 +3649,20 @@
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="66" t="s">
+      <c r="A12" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="B12" s="67"/>
-      <c r="C12" s="68"/>
-      <c r="D12" s="69" t="s">
+      <c r="B12" s="1"/>
+      <c r="C12" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D12" s="13" t="s">
         <v>430</v>
       </c>
-      <c r="E12" s="70">
+      <c r="E12" s="37">
         <v>129</v>
       </c>
-      <c r="F12" s="77" t="s">
+      <c r="F12" s="54" t="s">
         <v>557</v>
       </c>
       <c r="G12" s="21">
@@ -3660,7 +3672,7 @@
       <c r="H12" s="22"/>
       <c r="I12" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J12" s="24"/>
       <c r="K12" s="25"/>
@@ -17860,20 +17872,20 @@
       </c>
     </row>
     <row r="447" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A447" s="33" t="s">
+      <c r="A447" s="4" t="s">
         <v>496</v>
       </c>
-      <c r="B447" s="34" t="s">
-        <v>523</v>
-      </c>
-      <c r="C447" s="3"/>
-      <c r="D447" s="36" t="s">
+      <c r="B447" s="1"/>
+      <c r="C447" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D447" s="13" t="s">
         <v>803</v>
       </c>
-      <c r="E447" s="39">
+      <c r="E447" s="37">
         <v>9</v>
       </c>
-      <c r="F447" s="79" t="s">
+      <c r="F447" s="54" t="s">
         <v>796</v>
       </c>
       <c r="G447" s="21">
@@ -17883,7 +17895,7 @@
       <c r="H447" s="22"/>
       <c r="I447" s="23">
         <f t="shared" si="27"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J447" s="24"/>
       <c r="K447" s="25"/>

</xml_diff>